<commit_message>
menyelesaikan pembuatan chart, timeline, dan slice
</commit_message>
<xml_diff>
--- a/Analisis Retail Bisnis Omni-Channel.xlsx
+++ b/Analisis Retail Bisnis Omni-Channel.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aldy\Documents\DATA ANALYST\MICROSOFT EXCEL\PORTOFOLIO\Analisis Retail Bisnis Omni-Channel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BC05B65-0728-4592-AB0A-D73B78627A41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{587B3DA0-A944-43DE-A322-3B7B1E89898A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" firstSheet="1" activeTab="4" xr2:uid="{0FABD09F-C599-4D8F-AE1F-66CDC9C9D3DB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" firstSheet="1" activeTab="6" xr2:uid="{0FABD09F-C599-4D8F-AE1F-66CDC9C9D3DB}"/>
   </bookViews>
   <sheets>
     <sheet name="penjualan" sheetId="1" r:id="rId1"/>
@@ -23,18 +23,26 @@
   </sheets>
   <definedNames>
     <definedName name="NativeTimeline_Tanggal">#N/A</definedName>
+    <definedName name="Slicer_Kategori">#N/A</definedName>
+    <definedName name="Slicer_Kota">#N/A</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
     <pivotCache cacheId="0" r:id="rId8"/>
   </pivotCaches>
   <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
+      <x14:slicerCaches>
+        <x14:slicerCache r:id="rId9"/>
+        <x14:slicerCache r:id="rId10"/>
+      </x14:slicerCaches>
+    </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
       <x14:workbookPr/>
     </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}">
       <x15:timelineCacheRefs>
-        <x15:timelineCacheRef r:id="rId9"/>
+        <x15:timelineCacheRef r:id="rId11"/>
       </x15:timelineCacheRefs>
     </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -54,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2109" uniqueCount="595">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2116" uniqueCount="596">
   <si>
     <t>ID_Transaksi</t>
   </si>
@@ -1839,12 +1847,15 @@
   </si>
   <si>
     <t>Sum of Margin_Keuntungan</t>
+  </si>
+  <si>
+    <t>Sum of Laba_Kotor</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="_-[$Rp-3809]* #,##0_-;\-[$Rp-3809]* #,##0_-;_-[$Rp-3809]* &quot;-&quot;??_-;_-@_-"/>
@@ -2187,7 +2198,67 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="54">
+  <dxfs count="58">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <sz val="11"/>
+        <color theme="4" tint="-0.24994659260841701"/>
+        <name val="Poppins"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <sz val="8"/>
+        <color auto="1"/>
+        <name val="Poppins"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Poppins"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <sz val="8"/>
+        <color auto="1"/>
+        <name val="Poppins"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="0"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </left>
+        <right style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </right>
+        <top style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </top>
+        <bottom style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -3546,21 +3617,700 @@
       </border>
     </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="2" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="blue slicer style" pivot="0" table="0" count="6" xr9:uid="{95ABF258-362B-43FB-BEAC-4E4F6D81FFFE}">
+      <tableStyleElement type="wholeTable" dxfId="1"/>
+      <tableStyleElement type="headerRow" dxfId="0"/>
+    </tableStyle>
+    <tableStyle name="blue template" pivot="0" table="0" count="8" xr9:uid="{714AC691-FE5F-4B9C-9A2A-B9C5A38E8463}">
+      <tableStyleElement type="wholeTable" dxfId="3"/>
+      <tableStyleElement type="headerRow" dxfId="2"/>
+    </tableStyle>
+  </tableStyles>
   <colors>
     <mruColors>
+      <color rgb="FFFFFFA7"/>
       <color rgb="FF8C6047"/>
       <color rgb="FFFFFF9F"/>
-      <color rgb="FFFFFFA7"/>
       <color rgb="FFFFFF5D"/>
     </mruColors>
   </colors>
   <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{46F421CA-312F-682f-3DD2-61675219B42D}">
+      <x14:dxfs count="14">
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color theme="4" tint="-0.24994659260841701"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+          <fill>
+            <patternFill>
+              <bgColor theme="4" tint="0.59996337778862885"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color auto="1"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color theme="0"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+          <fill>
+            <patternFill>
+              <bgColor theme="4" tint="-0.24994659260841701"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color theme="0"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+          <fill>
+            <patternFill>
+              <bgColor theme="4" tint="-0.24994659260841701"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color auto="1"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color theme="0"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+          <fill>
+            <patternFill>
+              <bgColor theme="4" tint="-0.24994659260841701"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color theme="0"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+          <fill>
+            <patternFill>
+              <bgColor theme="4" tint="-0.24994659260841701"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color theme="0"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+          <fill>
+            <patternFill>
+              <bgColor theme="4" tint="-0.24994659260841701"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color auto="1"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color theme="4" tint="-0.24994659260841701"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color auto="1"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color theme="4" tint="-0.24994659260841701"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color auto="1"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color theme="4" tint="-0.24994659260841701"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+      </x14:dxfs>
+    </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1">
+        <x14:slicerStyle name="blue slicer style">
+          <x14:slicerStyleElements>
+            <x14:slicerStyleElement type="unselectedItemWithData" dxfId="3"/>
+            <x14:slicerStyleElement type="selectedItemWithData" dxfId="2"/>
+            <x14:slicerStyleElement type="selectedItemWithNoData" dxfId="1"/>
+            <x14:slicerStyleElement type="hoveredSelectedItemWithData" dxfId="0"/>
+          </x14:slicerStyleElements>
+        </x14:slicerStyle>
+      </x14:slicerStyles>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{A0A4C193-F2C1-4fcb-8827-314CF55A85BB}">
+      <x15:dxfs count="54">
+        <dxf>
+          <fill>
+            <patternFill patternType="solid">
+              <fgColor theme="0" tint="-0.14996795556505021"/>
+              <bgColor theme="4" tint="0.79998168889431442"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <fill>
+            <patternFill patternType="solid">
+              <fgColor theme="0"/>
+              <bgColor theme="4" tint="-0.24994659260841701"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color theme="4" tint="-0.24994659260841701"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="9"/>
+            <color auto="1"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color auto="1"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color theme="4" tint="-0.24994659260841701"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <fill>
+            <patternFill patternType="solid">
+              <fgColor theme="0" tint="-0.14999847407452621"/>
+              <bgColor theme="0" tint="-0.14999847407452621"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <fill>
+            <patternFill patternType="solid">
+              <fgColor theme="0"/>
+              <bgColor theme="4" tint="-0.24994659260841701"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color theme="4" tint="-0.24994659260841701"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="9"/>
+            <color auto="1"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color auto="1"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color theme="4" tint="-0.24994659260841701"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <fill>
+            <patternFill patternType="solid">
+              <fgColor theme="0" tint="-0.14999847407452621"/>
+              <bgColor theme="0" tint="-0.14999847407452621"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <fill>
+            <patternFill patternType="solid">
+              <fgColor theme="0"/>
+              <bgColor theme="4" tint="-0.24994659260841701"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color theme="4" tint="-0.24994659260841701"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="9"/>
+            <color auto="1"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color auto="1"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b val="0"/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color theme="4" tint="-0.24994659260841701"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <fill>
+            <patternFill patternType="solid">
+              <fgColor theme="0" tint="-0.14999847407452621"/>
+              <bgColor theme="0" tint="-0.14999847407452621"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <fill>
+            <patternFill patternType="solid">
+              <fgColor theme="0"/>
+              <bgColor theme="0"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color theme="4" tint="-0.24994659260841701"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="9"/>
+            <color auto="1"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color auto="1"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b val="0"/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color theme="4" tint="-0.24994659260841701"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <fill>
+            <patternFill patternType="solid">
+              <fgColor theme="0" tint="-0.14999847407452621"/>
+              <bgColor theme="0" tint="-0.14999847407452621"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <fill>
+            <patternFill patternType="solid">
+              <fgColor theme="0"/>
+              <bgColor theme="0"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="9"/>
+            <color auto="1"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="9"/>
+            <color auto="1"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color auto="1"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b val="0"/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color theme="4" tint="-0.24994659260841701"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <fill>
+            <patternFill patternType="solid">
+              <fgColor theme="0" tint="-0.14999847407452621"/>
+              <bgColor theme="0" tint="-0.14999847407452621"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <fill>
+            <patternFill patternType="solid">
+              <fgColor theme="0"/>
+              <bgColor theme="0"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <font>
+            <sz val="9"/>
+            <color theme="1" tint="0.499984740745262"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="9"/>
+            <color auto="1"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color auto="1"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b val="0"/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color theme="4" tint="-0.24994659260841701"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <fill>
+            <patternFill patternType="solid">
+              <fgColor theme="0" tint="-0.14999847407452621"/>
+              <bgColor theme="0" tint="-0.14999847407452621"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <fill>
+            <patternFill patternType="solid">
+              <fgColor theme="0"/>
+              <bgColor theme="0"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <font>
+            <sz val="9"/>
+            <color theme="1" tint="0.499984740745262"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <sz val="9"/>
+            <color theme="1" tint="0.499984740745262"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color auto="1"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b val="0"/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color theme="4" tint="-0.24994659260841701"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <fill>
+            <patternFill patternType="solid">
+              <fgColor theme="0" tint="-0.14999847407452621"/>
+              <bgColor theme="0" tint="-0.14999847407452621"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <fill>
+            <patternFill patternType="solid">
+              <fgColor theme="0"/>
+              <bgColor theme="0"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <font>
+            <sz val="9"/>
+            <color theme="1" tint="0.499984740745262"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <sz val="9"/>
+            <color theme="1" tint="0.499984740745262"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <sz val="11"/>
+            <color auto="1"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b val="0"/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color theme="4" tint="-0.24994659260841701"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+        <dxf>
+          <fill>
+            <patternFill patternType="solid">
+              <fgColor theme="0" tint="-0.14999847407452621"/>
+              <bgColor theme="0" tint="-0.14999847407452621"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <fill>
+            <patternFill patternType="solid">
+              <fgColor theme="0"/>
+              <bgColor theme="0"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <font>
+            <sz val="9"/>
+            <color theme="1" tint="0.499984740745262"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <sz val="9"/>
+            <color theme="1" tint="0.499984740745262"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <sz val="9"/>
+            <color theme="1" tint="0.499984740745262"/>
+          </font>
+        </dxf>
+        <dxf>
+          <font>
+            <b val="0"/>
+            <i val="0"/>
+            <sz val="8"/>
+            <color theme="4" tint="-0.24994659260841701"/>
+            <name val="Poppins"/>
+            <scheme val="none"/>
+          </font>
+        </dxf>
+      </x15:dxfs>
     </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1">
+        <x15:timelineStyle name="blue template">
+          <x15:timelineStyleElements>
+            <x15:timelineStyleElement type="selectionLabel" dxfId="5"/>
+            <x15:timelineStyleElement type="timeLevel" dxfId="4"/>
+            <x15:timelineStyleElement type="periodLabel1" dxfId="3"/>
+            <x15:timelineStyleElement type="periodLabel2" dxfId="2"/>
+            <x15:timelineStyleElement type="selectedTimeBlock" dxfId="1"/>
+            <x15:timelineStyleElement type="unselectedTimeBlock" dxfId="0"/>
+          </x15:timelineStyleElements>
+        </x15:timelineStyle>
+      </x15:timelineStyles>
     </ext>
   </extLst>
 </styleSheet>
@@ -3581,7 +4331,7 @@
   </mc:AlternateContent>
   <c:pivotSource>
     <c:name>[Analisis Retail Bisnis Omni-Channel.xlsx]analisis!analisis</c:name>
-    <c:fmtId val="0"/>
+    <c:fmtId val="11"/>
   </c:pivotSource>
   <c:chart>
     <c:title>
@@ -3661,7 +4411,9 @@
             <a:effectLst/>
           </c:spPr>
           <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
             <a:lstStyle/>
             <a:p>
               <a:pPr>
@@ -3691,10 +4443,13 @@
       <c:pivotFmt>
         <c:idx val="1"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent2">
-                <a:lumMod val="50000"/>
+                <a:lumMod val="75000"/>
               </a:schemeClr>
             </a:solidFill>
             <a:round/>
@@ -3714,7 +4469,232 @@
             <a:effectLst/>
           </c:spPr>
           <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="Poppins" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="Poppins" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1">
+              <a:lumMod val="75000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="Poppins" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="Poppins" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="3"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="28575" cap="rnd">
+            <a:solidFill>
+              <a:schemeClr val="accent2">
+                <a:lumMod val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="Poppins" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="Poppins" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="4"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1">
+              <a:lumMod val="75000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="Poppins" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="Poppins" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="5"/>
+        <c:spPr>
+          <a:ln w="28575" cap="rnd">
+            <a:solidFill>
+              <a:schemeClr val="accent2">
+                <a:lumMod val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
             <a:lstStyle/>
             <a:p>
               <a:pPr>
@@ -3804,26 +4784,26 @@
                 <c:formatCode>_-[$Rp-3809]* #,##0_-;\-[$Rp-3809]* #,##0_-;_-[$Rp-3809]* "-"??_-;_-@_-</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>567000000</c:v>
+                  <c:v>289800000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2676000000</c:v>
+                  <c:v>1260000000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>510000000</c:v>
+                  <c:v>261800000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1071000000</c:v>
+                  <c:v>512400000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>996200000</c:v>
+                  <c:v>489600000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-63F6-46B0-9AFF-3C647A8F7E08}"/>
+              <c16:uniqueId val="{00000000-1CD5-4064-BF41-FF9DC864A1DB}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3860,7 +4840,7 @@
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
                 <a:schemeClr val="accent2">
-                  <a:lumMod val="50000"/>
+                  <a:lumMod val="75000"/>
                 </a:schemeClr>
               </a:solidFill>
               <a:round/>
@@ -3900,19 +4880,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>29.245275888133023</c:v>
+                  <c:v>14.017054043839757</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>22.367766203703731</c:v>
+                  <c:v>10.844340277777777</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>24.156746031746</c:v>
+                  <c:v>12.644491129785242</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>30.3317507558579</c:v>
+                  <c:v>14.975907029478458</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>24.34109477124181</c:v>
+                  <c:v>12.231413398692801</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3920,7 +4900,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-63F6-46B0-9AFF-3C647A8F7E08}"/>
+              <c16:uniqueId val="{00000001-1CD5-4064-BF41-FF9DC864A1DB}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4255,7 +5235,822 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[Analisis Retail Bisnis Omni-Channel.xlsx]analisis!PivotTable1</c:name>
+    <c:fmtId val="14"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1100" b="1">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Poppins" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+                <a:cs typeface="Poppins" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+              </a:rPr>
+              <a:t>Kontribusi</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Poppins" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+                <a:cs typeface="Poppins" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+              </a:rPr>
+              <a:t> Laba  Per Kota</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Poppins" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+              <a:cs typeface="Poppins" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+            </a:endParaRPr>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="800" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="bg1"/>
+                  </a:solidFill>
+                  <a:latin typeface="Poppins" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="Poppins" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="1"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1">
+              <a:lumMod val="75000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1">
+              <a:lumMod val="60000"/>
+              <a:lumOff val="40000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="3"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent2">
+              <a:lumMod val="75000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="4"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent2">
+              <a:lumMod val="60000"/>
+              <a:lumOff val="40000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="5"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="800" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="bg1"/>
+                  </a:solidFill>
+                  <a:latin typeface="Poppins" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="Poppins" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="1"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="6"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1">
+              <a:lumMod val="75000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="7"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1">
+              <a:lumMod val="60000"/>
+              <a:lumOff val="40000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="8"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent2">
+              <a:lumMod val="60000"/>
+              <a:lumOff val="40000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="9"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent2">
+              <a:lumMod val="75000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="10"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="800" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="bg1"/>
+                  </a:solidFill>
+                  <a:latin typeface="Poppins" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="Poppins" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="1"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="11"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1">
+              <a:lumMod val="75000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="12"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1">
+              <a:lumMod val="60000"/>
+              <a:lumOff val="40000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="13"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent2">
+              <a:lumMod val="60000"/>
+              <a:lumOff val="40000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="14"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent2">
+              <a:lumMod val="75000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>analisis!$G$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-39AD-4074-A2BD-0AD721C29F98}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
+                  <a:lumOff val="40000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-39AD-4074-A2BD-0AD721C29F98}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="60000"/>
+                  <a:lumOff val="40000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-39AD-4074-A2BD-0AD721C29F98}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000007-39AD-4074-A2BD-0AD721C29F98}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="800" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="bg1"/>
+                    </a:solidFill>
+                    <a:latin typeface="Poppins" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="Poppins" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="1"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="1"/>
+            <c:leaderLines>
+              <c:spPr>
+                <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="35000"/>
+                      <a:lumOff val="65000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:round/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+            </c:leaderLines>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>analisis!$F$4:$F$8</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Jakarta</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Makassar</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Medan</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Surabaya</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>analisis!$G$4:$G$8</c:f>
+              <c:numCache>
+                <c:formatCode>_-[$Rp-3809]* #,##0_-;\-[$Rp-3809]* #,##0_-;_-[$Rp-3809]* "-"??_-;_-@_-</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>167845000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>111475000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>234065000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>120440000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000008-39AD-4074-A2BD-0AD721C29F98}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="1"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Poppins" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="Poppins" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+        <c14:dropZoneSeries val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -4811,31 +6606,552 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>781050</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
+      <xdr:rowOff>127907</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>49306</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>146957</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1">
+        <xdr:cNvPr id="4" name="Chart 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0580262D-F0D7-6767-4290-2A419F72E9FE}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C090A6E6-249C-44AC-9A37-C7F4CD99B2A3}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="0"/>
@@ -4851,25 +7167,25 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1333500</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>13607</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>10294</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>352425</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>140922</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:tsle="http://schemas.microsoft.com/office/drawing/2012/timeslicer" Requires="tsle">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
-            <xdr:cNvPr id="3" name="Tanggal">
+            <xdr:cNvPr id="5" name="Tanggal">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3366D860-08CA-BAEF-5F57-FA87A974B644}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C8ADB4C4-D361-43E5-9AE8-93E003C4D02A}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -4896,8 +7212,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="1333500" y="1962150"/>
-              <a:ext cx="5581650" cy="1371600"/>
+              <a:off x="92048" y="2722118"/>
+              <a:ext cx="6116011" cy="1363275"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -4918,6 +7234,200 @@
               <a:r>
                 <a:rPr lang="en-ID" sz="1100"/>
                 <a:t>Timeline: Works in Excel 2013 or higher. Do not move or resize.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>502425</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>178253</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>454800</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>197303</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Chart 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ED53858A-7BA1-4F93-B9C3-7160E6394346}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>210911</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>89809</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>399089</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>51707</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="7" name="Kota">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{64B326E5-1A96-4AEE-A94F-D468B5FD1846}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
+              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="Kota"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="894470" y="7732221"/>
+              <a:ext cx="2687090" cy="948015"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-ID" sz="1100"/>
+                <a:t>This shape represents a slicer. Slicers are supported in Excel 2010 or later.
+If the shape was modified in an earlier version of Excel, or if the workbook was saved in Excel 2003 or earlier, the slicer cannot be used.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>264378</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>62594</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>50107</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>21772</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="8" name="Kategori">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{29F731CD-373D-4D7A-A5C0-58845854EEDE}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
+              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="Kategori"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="4051966" y="7705006"/>
+              <a:ext cx="2206200" cy="1191825"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-ID" sz="1100"/>
+                <a:t>This shape represents a slicer. Slicers are supported in Excel 2010 or later.
+If the shape was modified in an earlier version of Excel, or if the workbook was saved in Excel 2003 or earlier, the slicer cannot be used.</a:t>
               </a:r>
             </a:p>
           </xdr:txBody>
@@ -15901,7 +18411,1217 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{33554939-956D-4BE9-A88C-42E3B53823EE}" name="analisis" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="3">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{240C8AC7-0F61-4DDD-9013-EAC85AE6134F}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="15">
+  <location ref="F3:G8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="20">
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" numFmtId="164" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="364">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item x="30"/>
+        <item x="31"/>
+        <item x="32"/>
+        <item x="33"/>
+        <item x="34"/>
+        <item x="35"/>
+        <item x="36"/>
+        <item x="37"/>
+        <item x="38"/>
+        <item x="39"/>
+        <item x="40"/>
+        <item x="41"/>
+        <item x="42"/>
+        <item x="43"/>
+        <item x="44"/>
+        <item x="45"/>
+        <item x="46"/>
+        <item x="47"/>
+        <item x="48"/>
+        <item x="49"/>
+        <item x="50"/>
+        <item x="51"/>
+        <item x="52"/>
+        <item x="53"/>
+        <item x="54"/>
+        <item x="55"/>
+        <item x="56"/>
+        <item x="57"/>
+        <item x="58"/>
+        <item x="59"/>
+        <item x="60"/>
+        <item x="61"/>
+        <item x="62"/>
+        <item x="63"/>
+        <item x="64"/>
+        <item x="65"/>
+        <item x="66"/>
+        <item x="67"/>
+        <item x="68"/>
+        <item x="69"/>
+        <item x="70"/>
+        <item x="71"/>
+        <item x="72"/>
+        <item x="73"/>
+        <item x="74"/>
+        <item x="75"/>
+        <item x="76"/>
+        <item x="77"/>
+        <item x="78"/>
+        <item x="79"/>
+        <item x="80"/>
+        <item x="81"/>
+        <item x="82"/>
+        <item x="83"/>
+        <item x="84"/>
+        <item x="85"/>
+        <item x="86"/>
+        <item x="87"/>
+        <item x="88"/>
+        <item x="89"/>
+        <item x="90"/>
+        <item x="91"/>
+        <item x="92"/>
+        <item x="93"/>
+        <item x="94"/>
+        <item x="95"/>
+        <item x="96"/>
+        <item x="97"/>
+        <item x="98"/>
+        <item x="99"/>
+        <item x="100"/>
+        <item x="101"/>
+        <item x="102"/>
+        <item x="103"/>
+        <item x="104"/>
+        <item x="105"/>
+        <item x="106"/>
+        <item x="107"/>
+        <item x="108"/>
+        <item x="109"/>
+        <item x="110"/>
+        <item x="111"/>
+        <item x="112"/>
+        <item x="113"/>
+        <item x="114"/>
+        <item x="115"/>
+        <item x="116"/>
+        <item x="117"/>
+        <item x="118"/>
+        <item x="119"/>
+        <item x="120"/>
+        <item x="121"/>
+        <item x="122"/>
+        <item x="123"/>
+        <item x="124"/>
+        <item x="125"/>
+        <item x="126"/>
+        <item x="127"/>
+        <item x="128"/>
+        <item x="129"/>
+        <item x="130"/>
+        <item x="131"/>
+        <item x="132"/>
+        <item x="133"/>
+        <item x="134"/>
+        <item x="135"/>
+        <item x="136"/>
+        <item x="137"/>
+        <item x="138"/>
+        <item x="139"/>
+        <item x="140"/>
+        <item x="141"/>
+        <item x="142"/>
+        <item x="143"/>
+        <item x="144"/>
+        <item x="145"/>
+        <item x="146"/>
+        <item x="147"/>
+        <item x="148"/>
+        <item x="149"/>
+        <item x="150"/>
+        <item x="151"/>
+        <item x="152"/>
+        <item x="153"/>
+        <item x="154"/>
+        <item x="155"/>
+        <item x="156"/>
+        <item x="157"/>
+        <item x="158"/>
+        <item x="159"/>
+        <item x="160"/>
+        <item x="161"/>
+        <item x="162"/>
+        <item x="163"/>
+        <item x="164"/>
+        <item x="165"/>
+        <item x="166"/>
+        <item x="167"/>
+        <item x="168"/>
+        <item x="169"/>
+        <item x="170"/>
+        <item x="171"/>
+        <item x="172"/>
+        <item x="173"/>
+        <item x="174"/>
+        <item x="175"/>
+        <item x="176"/>
+        <item x="177"/>
+        <item x="178"/>
+        <item x="179"/>
+        <item x="180"/>
+        <item x="181"/>
+        <item x="182"/>
+        <item x="183"/>
+        <item x="184"/>
+        <item x="185"/>
+        <item x="186"/>
+        <item x="187"/>
+        <item x="188"/>
+        <item x="189"/>
+        <item x="190"/>
+        <item x="191"/>
+        <item x="192"/>
+        <item x="193"/>
+        <item x="194"/>
+        <item x="195"/>
+        <item x="196"/>
+        <item x="197"/>
+        <item x="198"/>
+        <item x="199"/>
+        <item x="200"/>
+        <item x="201"/>
+        <item x="202"/>
+        <item x="203"/>
+        <item x="204"/>
+        <item x="205"/>
+        <item x="206"/>
+        <item x="207"/>
+        <item x="208"/>
+        <item x="209"/>
+        <item x="210"/>
+        <item x="211"/>
+        <item x="212"/>
+        <item x="213"/>
+        <item x="214"/>
+        <item x="215"/>
+        <item x="216"/>
+        <item x="217"/>
+        <item x="218"/>
+        <item x="219"/>
+        <item x="220"/>
+        <item x="221"/>
+        <item x="222"/>
+        <item x="223"/>
+        <item x="224"/>
+        <item x="225"/>
+        <item x="226"/>
+        <item x="227"/>
+        <item x="228"/>
+        <item x="229"/>
+        <item x="230"/>
+        <item x="231"/>
+        <item x="232"/>
+        <item x="233"/>
+        <item x="234"/>
+        <item x="235"/>
+        <item x="236"/>
+        <item x="237"/>
+        <item x="238"/>
+        <item x="239"/>
+        <item x="240"/>
+        <item x="241"/>
+        <item x="242"/>
+        <item x="243"/>
+        <item x="244"/>
+        <item x="245"/>
+        <item x="246"/>
+        <item x="247"/>
+        <item x="248"/>
+        <item x="249"/>
+        <item x="250"/>
+        <item x="251"/>
+        <item x="252"/>
+        <item x="253"/>
+        <item x="254"/>
+        <item x="255"/>
+        <item x="256"/>
+        <item x="257"/>
+        <item x="258"/>
+        <item x="259"/>
+        <item x="260"/>
+        <item x="261"/>
+        <item x="262"/>
+        <item x="263"/>
+        <item x="264"/>
+        <item x="265"/>
+        <item x="266"/>
+        <item x="267"/>
+        <item x="268"/>
+        <item x="269"/>
+        <item x="270"/>
+        <item x="271"/>
+        <item x="272"/>
+        <item x="273"/>
+        <item x="274"/>
+        <item x="275"/>
+        <item x="276"/>
+        <item x="277"/>
+        <item x="278"/>
+        <item x="279"/>
+        <item x="280"/>
+        <item x="281"/>
+        <item x="282"/>
+        <item x="283"/>
+        <item x="284"/>
+        <item x="285"/>
+        <item x="286"/>
+        <item x="287"/>
+        <item x="288"/>
+        <item x="289"/>
+        <item x="290"/>
+        <item x="291"/>
+        <item x="292"/>
+        <item x="293"/>
+        <item x="294"/>
+        <item x="295"/>
+        <item x="296"/>
+        <item x="297"/>
+        <item x="298"/>
+        <item x="299"/>
+        <item x="300"/>
+        <item x="301"/>
+        <item x="302"/>
+        <item x="303"/>
+        <item x="304"/>
+        <item x="305"/>
+        <item x="306"/>
+        <item x="307"/>
+        <item x="308"/>
+        <item x="309"/>
+        <item x="310"/>
+        <item x="311"/>
+        <item x="312"/>
+        <item x="313"/>
+        <item x="314"/>
+        <item x="315"/>
+        <item x="316"/>
+        <item x="317"/>
+        <item x="318"/>
+        <item x="319"/>
+        <item x="320"/>
+        <item x="321"/>
+        <item x="322"/>
+        <item x="323"/>
+        <item x="324"/>
+        <item x="325"/>
+        <item x="326"/>
+        <item x="327"/>
+        <item x="328"/>
+        <item x="329"/>
+        <item x="330"/>
+        <item x="331"/>
+        <item x="332"/>
+        <item x="333"/>
+        <item x="334"/>
+        <item x="335"/>
+        <item x="336"/>
+        <item x="337"/>
+        <item x="338"/>
+        <item x="339"/>
+        <item x="340"/>
+        <item x="341"/>
+        <item x="342"/>
+        <item x="343"/>
+        <item x="344"/>
+        <item x="345"/>
+        <item x="346"/>
+        <item x="347"/>
+        <item x="348"/>
+        <item x="349"/>
+        <item x="350"/>
+        <item x="351"/>
+        <item x="352"/>
+        <item x="353"/>
+        <item x="354"/>
+        <item x="355"/>
+        <item x="356"/>
+        <item x="357"/>
+        <item x="358"/>
+        <item x="359"/>
+        <item x="360"/>
+        <item x="361"/>
+        <item x="362"/>
+        <item x="363"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="1"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="5">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="3"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="3">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="2"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" numFmtId="165" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" numFmtId="165" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" numFmtId="165" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" numFmtId="166" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" numFmtId="165" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" numFmtId="165" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" numFmtId="165" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" numFmtId="165" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField dataField="1" compact="0" numFmtId="165" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="98">
+        <item x="61"/>
+        <item x="48"/>
+        <item x="26"/>
+        <item x="78"/>
+        <item x="90"/>
+        <item x="29"/>
+        <item x="42"/>
+        <item x="33"/>
+        <item x="52"/>
+        <item x="1"/>
+        <item x="23"/>
+        <item x="6"/>
+        <item x="54"/>
+        <item x="32"/>
+        <item x="9"/>
+        <item x="69"/>
+        <item x="92"/>
+        <item x="21"/>
+        <item x="93"/>
+        <item x="39"/>
+        <item x="2"/>
+        <item x="36"/>
+        <item x="41"/>
+        <item x="27"/>
+        <item x="85"/>
+        <item x="44"/>
+        <item x="13"/>
+        <item x="31"/>
+        <item x="37"/>
+        <item x="35"/>
+        <item x="73"/>
+        <item x="46"/>
+        <item x="51"/>
+        <item x="68"/>
+        <item x="76"/>
+        <item x="66"/>
+        <item x="65"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="57"/>
+        <item x="96"/>
+        <item x="16"/>
+        <item x="83"/>
+        <item x="17"/>
+        <item x="19"/>
+        <item x="3"/>
+        <item x="22"/>
+        <item x="88"/>
+        <item x="14"/>
+        <item x="59"/>
+        <item x="8"/>
+        <item x="47"/>
+        <item x="64"/>
+        <item x="70"/>
+        <item x="15"/>
+        <item x="82"/>
+        <item x="56"/>
+        <item x="72"/>
+        <item x="89"/>
+        <item x="18"/>
+        <item x="87"/>
+        <item x="55"/>
+        <item x="62"/>
+        <item x="43"/>
+        <item x="4"/>
+        <item x="67"/>
+        <item x="60"/>
+        <item x="50"/>
+        <item x="86"/>
+        <item x="79"/>
+        <item x="10"/>
+        <item x="5"/>
+        <item x="49"/>
+        <item x="7"/>
+        <item x="80"/>
+        <item x="77"/>
+        <item x="24"/>
+        <item x="97"/>
+        <item x="95"/>
+        <item x="0"/>
+        <item x="28"/>
+        <item x="71"/>
+        <item x="63"/>
+        <item x="74"/>
+        <item x="38"/>
+        <item x="94"/>
+        <item x="20"/>
+        <item x="45"/>
+        <item x="25"/>
+        <item x="34"/>
+        <item x="53"/>
+        <item x="81"/>
+        <item x="40"/>
+        <item x="30"/>
+        <item x="58"/>
+        <item x="75"/>
+        <item x="84"/>
+        <item x="91"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="20">
+        <item x="13"/>
+        <item x="15"/>
+        <item x="6"/>
+        <item x="9"/>
+        <item x="17"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item x="11"/>
+        <item x="19"/>
+        <item x="7"/>
+        <item x="10"/>
+        <item x="5"/>
+        <item x="8"/>
+        <item x="12"/>
+        <item x="4"/>
+        <item x="18"/>
+        <item x="16"/>
+        <item x="2"/>
+        <item x="14"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0" defaultSubtotal="0">
+      <items count="368">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item x="30"/>
+        <item x="31"/>
+        <item x="32"/>
+        <item x="33"/>
+        <item x="34"/>
+        <item x="35"/>
+        <item x="36"/>
+        <item x="37"/>
+        <item x="38"/>
+        <item x="39"/>
+        <item x="40"/>
+        <item x="41"/>
+        <item x="42"/>
+        <item x="43"/>
+        <item x="44"/>
+        <item x="45"/>
+        <item x="46"/>
+        <item x="47"/>
+        <item x="48"/>
+        <item x="49"/>
+        <item x="50"/>
+        <item x="51"/>
+        <item x="52"/>
+        <item x="53"/>
+        <item x="54"/>
+        <item x="55"/>
+        <item x="56"/>
+        <item x="57"/>
+        <item x="58"/>
+        <item x="59"/>
+        <item x="60"/>
+        <item x="61"/>
+        <item x="62"/>
+        <item x="63"/>
+        <item x="64"/>
+        <item x="65"/>
+        <item x="66"/>
+        <item x="67"/>
+        <item x="68"/>
+        <item x="69"/>
+        <item x="70"/>
+        <item x="71"/>
+        <item x="72"/>
+        <item x="73"/>
+        <item x="74"/>
+        <item x="75"/>
+        <item x="76"/>
+        <item x="77"/>
+        <item x="78"/>
+        <item x="79"/>
+        <item x="80"/>
+        <item x="81"/>
+        <item x="82"/>
+        <item x="83"/>
+        <item x="84"/>
+        <item x="85"/>
+        <item x="86"/>
+        <item x="87"/>
+        <item x="88"/>
+        <item x="89"/>
+        <item x="90"/>
+        <item x="91"/>
+        <item x="92"/>
+        <item x="93"/>
+        <item x="94"/>
+        <item x="95"/>
+        <item x="96"/>
+        <item x="97"/>
+        <item x="98"/>
+        <item x="99"/>
+        <item x="100"/>
+        <item x="101"/>
+        <item x="102"/>
+        <item x="103"/>
+        <item x="104"/>
+        <item x="105"/>
+        <item x="106"/>
+        <item x="107"/>
+        <item x="108"/>
+        <item x="109"/>
+        <item x="110"/>
+        <item x="111"/>
+        <item x="112"/>
+        <item x="113"/>
+        <item x="114"/>
+        <item x="115"/>
+        <item x="116"/>
+        <item x="117"/>
+        <item x="118"/>
+        <item x="119"/>
+        <item x="120"/>
+        <item x="121"/>
+        <item x="122"/>
+        <item x="123"/>
+        <item x="124"/>
+        <item x="125"/>
+        <item x="126"/>
+        <item x="127"/>
+        <item x="128"/>
+        <item x="129"/>
+        <item x="130"/>
+        <item x="131"/>
+        <item x="132"/>
+        <item x="133"/>
+        <item x="134"/>
+        <item x="135"/>
+        <item x="136"/>
+        <item x="137"/>
+        <item x="138"/>
+        <item x="139"/>
+        <item x="140"/>
+        <item x="141"/>
+        <item x="142"/>
+        <item x="143"/>
+        <item x="144"/>
+        <item x="145"/>
+        <item x="146"/>
+        <item x="147"/>
+        <item x="148"/>
+        <item x="149"/>
+        <item x="150"/>
+        <item x="151"/>
+        <item x="152"/>
+        <item x="153"/>
+        <item x="154"/>
+        <item x="155"/>
+        <item x="156"/>
+        <item x="157"/>
+        <item x="158"/>
+        <item x="159"/>
+        <item x="160"/>
+        <item x="161"/>
+        <item x="162"/>
+        <item x="163"/>
+        <item x="164"/>
+        <item x="165"/>
+        <item x="166"/>
+        <item x="167"/>
+        <item x="168"/>
+        <item x="169"/>
+        <item x="170"/>
+        <item x="171"/>
+        <item x="172"/>
+        <item x="173"/>
+        <item x="174"/>
+        <item x="175"/>
+        <item x="176"/>
+        <item x="177"/>
+        <item x="178"/>
+        <item x="179"/>
+        <item x="180"/>
+        <item x="181"/>
+        <item x="182"/>
+        <item x="183"/>
+        <item x="184"/>
+        <item x="185"/>
+        <item x="186"/>
+        <item x="187"/>
+        <item x="188"/>
+        <item x="189"/>
+        <item x="190"/>
+        <item x="191"/>
+        <item x="192"/>
+        <item x="193"/>
+        <item x="194"/>
+        <item x="195"/>
+        <item x="196"/>
+        <item x="197"/>
+        <item x="198"/>
+        <item x="199"/>
+        <item x="200"/>
+        <item x="201"/>
+        <item x="202"/>
+        <item x="203"/>
+        <item x="204"/>
+        <item x="205"/>
+        <item x="206"/>
+        <item x="207"/>
+        <item x="208"/>
+        <item x="209"/>
+        <item x="210"/>
+        <item x="211"/>
+        <item x="212"/>
+        <item x="213"/>
+        <item x="214"/>
+        <item x="215"/>
+        <item x="216"/>
+        <item x="217"/>
+        <item x="218"/>
+        <item x="219"/>
+        <item x="220"/>
+        <item x="221"/>
+        <item x="222"/>
+        <item x="223"/>
+        <item x="224"/>
+        <item x="225"/>
+        <item x="226"/>
+        <item x="227"/>
+        <item x="228"/>
+        <item x="229"/>
+        <item x="230"/>
+        <item x="231"/>
+        <item x="232"/>
+        <item x="233"/>
+        <item x="234"/>
+        <item x="235"/>
+        <item x="236"/>
+        <item x="237"/>
+        <item x="238"/>
+        <item x="239"/>
+        <item x="240"/>
+        <item x="241"/>
+        <item x="242"/>
+        <item x="243"/>
+        <item x="244"/>
+        <item x="245"/>
+        <item x="246"/>
+        <item x="247"/>
+        <item x="248"/>
+        <item x="249"/>
+        <item x="250"/>
+        <item x="251"/>
+        <item x="252"/>
+        <item x="253"/>
+        <item x="254"/>
+        <item x="255"/>
+        <item x="256"/>
+        <item x="257"/>
+        <item x="258"/>
+        <item x="259"/>
+        <item x="260"/>
+        <item x="261"/>
+        <item x="262"/>
+        <item x="263"/>
+        <item x="264"/>
+        <item x="265"/>
+        <item x="266"/>
+        <item x="267"/>
+        <item x="268"/>
+        <item x="269"/>
+        <item x="270"/>
+        <item x="271"/>
+        <item x="272"/>
+        <item x="273"/>
+        <item x="274"/>
+        <item x="275"/>
+        <item x="276"/>
+        <item x="277"/>
+        <item x="278"/>
+        <item x="279"/>
+        <item x="280"/>
+        <item x="281"/>
+        <item x="282"/>
+        <item x="283"/>
+        <item x="284"/>
+        <item x="285"/>
+        <item x="286"/>
+        <item x="287"/>
+        <item x="288"/>
+        <item x="289"/>
+        <item x="290"/>
+        <item x="291"/>
+        <item x="292"/>
+        <item x="293"/>
+        <item x="294"/>
+        <item x="295"/>
+        <item x="296"/>
+        <item x="297"/>
+        <item x="298"/>
+        <item x="299"/>
+        <item x="300"/>
+        <item x="301"/>
+        <item x="302"/>
+        <item x="303"/>
+        <item x="304"/>
+        <item x="305"/>
+        <item x="306"/>
+        <item x="307"/>
+        <item x="308"/>
+        <item x="309"/>
+        <item x="310"/>
+        <item x="311"/>
+        <item x="312"/>
+        <item x="313"/>
+        <item x="314"/>
+        <item x="315"/>
+        <item x="316"/>
+        <item x="317"/>
+        <item x="318"/>
+        <item x="319"/>
+        <item x="320"/>
+        <item x="321"/>
+        <item x="322"/>
+        <item x="323"/>
+        <item x="324"/>
+        <item x="325"/>
+        <item x="326"/>
+        <item x="327"/>
+        <item x="328"/>
+        <item x="329"/>
+        <item x="330"/>
+        <item x="331"/>
+        <item x="332"/>
+        <item x="333"/>
+        <item x="334"/>
+        <item x="335"/>
+        <item x="336"/>
+        <item x="337"/>
+        <item x="338"/>
+        <item x="339"/>
+        <item x="340"/>
+        <item x="341"/>
+        <item x="342"/>
+        <item x="343"/>
+        <item x="344"/>
+        <item x="345"/>
+        <item x="346"/>
+        <item x="347"/>
+        <item x="348"/>
+        <item x="349"/>
+        <item x="350"/>
+        <item x="351"/>
+        <item x="352"/>
+        <item x="353"/>
+        <item x="354"/>
+        <item x="355"/>
+        <item x="356"/>
+        <item x="357"/>
+        <item x="358"/>
+        <item x="359"/>
+        <item x="360"/>
+        <item x="361"/>
+        <item x="362"/>
+        <item x="363"/>
+        <item x="364"/>
+        <item x="365"/>
+        <item x="366"/>
+        <item x="367"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0" defaultSubtotal="0">
+      <items count="14">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Laba_Kotor" fld="16" baseField="0" baseItem="0" numFmtId="165"/>
+  </dataFields>
+  <chartFormats count="20">
+    <chartFormat chart="9" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="9" format="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="9" format="2">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="9" format="3">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="9" format="4">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="12" format="5" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="12" format="6">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="12" format="7">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="12" format="8">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="12" format="9">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="13" format="10" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="13" format="11">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="13" format="12">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="13" format="13">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="13" format="14">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="14" format="10" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="14" format="11">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="14" format="12">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="14" format="13">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="14" format="14">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <filters count="1">
+    <filter fld="1" type="dateBetween" evalOrder="-1" id="21" name="Tanggal">
+      <autoFilter ref="A1">
+        <filterColumn colId="0">
+          <customFilters and="1">
+            <customFilter operator="greaterThanOrEqual" val="45689"/>
+            <customFilter operator="lessThanOrEqual" val="45869"/>
+          </customFilters>
+        </filterColumn>
+      </autoFilter>
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{0605FD5F-26C8-4aeb-8148-2DB25E43C511}">
+          <x15:pivotFilter useWholeDay="1"/>
+        </ext>
+      </extLst>
+    </filter>
+  </filters>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{33554939-956D-4BE9-A88C-42E3B53823EE}" name="analisis" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="12">
   <location ref="A3:C9" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="20">
     <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
@@ -16863,7 +20583,7 @@
     <dataField name="Sum of Total_Pendapatan_Kotor" fld="12" baseField="0" baseItem="0" numFmtId="165"/>
     <dataField name="Sum of Margin_Keuntungan" fld="17" baseField="0" baseItem="0"/>
   </dataFields>
-  <chartFormats count="4">
+  <chartFormats count="12">
     <chartFormat chart="0" format="0" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
@@ -16882,32 +20602,115 @@
         </references>
       </pivotArea>
     </chartFormat>
-    <chartFormat chart="0" format="2">
+    <chartFormat chart="4" format="2" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
+        <references count="1">
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="4"/>
           </reference>
         </references>
       </pivotArea>
     </chartFormat>
-    <chartFormat chart="0" format="3">
+    <chartFormat chart="4" format="3" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
+        <references count="1">
           <reference field="4294967294" count="1" selected="0">
             <x v="1"/>
           </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="4"/>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="5" format="4" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="5" format="5" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="9" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="9" format="3" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="10" format="4" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="10" format="5" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="11" format="4" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="11" format="5" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
           </reference>
         </references>
       </pivotArea>
     </chartFormat>
   </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <filters count="1">
+    <filter fld="1" type="dateBetween" evalOrder="-1" id="21" name="Tanggal">
+      <autoFilter ref="A1">
+        <filterColumn colId="0">
+          <customFilters and="1">
+            <customFilter operator="greaterThanOrEqual" val="45689"/>
+            <customFilter operator="lessThanOrEqual" val="45869"/>
+          </customFilters>
+        </filterColumn>
+      </autoFilter>
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{0605FD5F-26C8-4aeb-8148-2DB25E43C511}">
+          <x15:pivotFilter useWholeDay="1"/>
+        </ext>
+      </extLst>
+    </filter>
+  </filters>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
       <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
@@ -16919,50 +20722,92 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/slicerCaches/slicerCache1.xml><?xml version="1.0" encoding="utf-8"?>
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Kota" xr10:uid="{778F3C14-16CE-40F3-B5D6-56003E13C63D}" sourceName="Kota">
+  <pivotTables>
+    <pivotTable tabId="6" name="analisis"/>
+  </pivotTables>
+  <data>
+    <tabular pivotCacheId="241815905">
+      <items count="4">
+        <i x="0" s="1"/>
+        <i x="3" s="1"/>
+        <i x="2" s="1"/>
+        <i x="1" s="1"/>
+      </items>
+    </tabular>
+  </data>
+</slicerCacheDefinition>
+</file>
+
+<file path=xl/slicerCaches/slicerCache2.xml><?xml version="1.0" encoding="utf-8"?>
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Kategori" xr10:uid="{3A4EE724-4778-4E2C-98B6-A2758514889C}" sourceName="Kategori">
+  <pivotTables>
+    <pivotTable tabId="6" name="analisis"/>
+  </pivotTables>
+  <data>
+    <tabular pivotCacheId="241815905">
+      <items count="3">
+        <i x="1" s="1"/>
+        <i x="0" s="1"/>
+        <i x="2" s="1"/>
+      </items>
+    </tabular>
+  </data>
+</slicerCacheDefinition>
+</file>
+
+<file path=xl/slicers/slicer1.xml><?xml version="1.0" encoding="utf-8"?>
+<slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
+  <slicer name="Kota" xr10:uid="{2F14FB20-EA99-479D-BF43-71C5B0CBE7C0}" cache="Slicer_Kota" caption="Kota" columnCount="2" style="blue slicer style" rowHeight="241300"/>
+  <slicer name="Kategori" xr10:uid="{0AD13CFD-B6F7-43DC-A11D-7BC70C551F06}" cache="Slicer_Kategori" caption="Kategori" style="blue slicer style" rowHeight="241300"/>
+</slicers>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{91C63E51-A52D-46AB-91EB-CF63578A5333}" name="Table1" displayName="Table1" ref="A1:R501" totalsRowShown="0" headerRowDxfId="53" dataDxfId="51" headerRowBorderDxfId="52" tableBorderDxfId="50" totalsRowBorderDxfId="49">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{91C63E51-A52D-46AB-91EB-CF63578A5333}" name="Table1" displayName="Table1" ref="A1:R501" totalsRowShown="0" headerRowDxfId="57" dataDxfId="55" headerRowBorderDxfId="56" tableBorderDxfId="54" totalsRowBorderDxfId="53">
   <autoFilter ref="A1:R501" xr:uid="{91C63E51-A52D-46AB-91EB-CF63578A5333}"/>
   <tableColumns count="18">
-    <tableColumn id="1" xr3:uid="{535352A0-284A-4EC3-BEA5-FCAC4589AD45}" name="ID_Transaksi" dataDxfId="48"/>
-    <tableColumn id="2" xr3:uid="{60F5C6B6-2EE4-4C37-834D-803292CD8C49}" name="Tanggal" dataDxfId="47"/>
-    <tableColumn id="3" xr3:uid="{E56A6511-4721-46F1-A464-627EE6ED25E5}" name="Kota" dataDxfId="46"/>
-    <tableColumn id="4" xr3:uid="{D6C78C85-4803-494C-B4E3-8459D877E28E}" name="SKU" dataDxfId="45"/>
-    <tableColumn id="5" xr3:uid="{0C6A6903-F5CE-4107-9FDE-CC53F5F04204}" name="Jumlah_Unit" dataDxfId="44"/>
-    <tableColumn id="6" xr3:uid="{048E2C98-E916-4C7C-AA4A-3150159A27E8}" name="Kode_Promo" dataDxfId="43"/>
-    <tableColumn id="7" xr3:uid="{3B8F5B69-10F0-4AEE-8CCF-65814EF6B3D8}" name="Nama_Produk" dataDxfId="42">
+    <tableColumn id="1" xr3:uid="{535352A0-284A-4EC3-BEA5-FCAC4589AD45}" name="ID_Transaksi" dataDxfId="52"/>
+    <tableColumn id="2" xr3:uid="{60F5C6B6-2EE4-4C37-834D-803292CD8C49}" name="Tanggal" dataDxfId="51"/>
+    <tableColumn id="3" xr3:uid="{E56A6511-4721-46F1-A464-627EE6ED25E5}" name="Kota" dataDxfId="50"/>
+    <tableColumn id="4" xr3:uid="{D6C78C85-4803-494C-B4E3-8459D877E28E}" name="SKU" dataDxfId="49"/>
+    <tableColumn id="5" xr3:uid="{0C6A6903-F5CE-4107-9FDE-CC53F5F04204}" name="Jumlah_Unit" dataDxfId="48"/>
+    <tableColumn id="6" xr3:uid="{048E2C98-E916-4C7C-AA4A-3150159A27E8}" name="Kode_Promo" dataDxfId="47"/>
+    <tableColumn id="7" xr3:uid="{3B8F5B69-10F0-4AEE-8CCF-65814EF6B3D8}" name="Nama_Produk" dataDxfId="46">
       <calculatedColumnFormula>INDEX(Table2[Nama Produk],MATCH(Table1[[#This Row],[SKU]],Table2[SKU],0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{735DE14D-F3A8-4241-B953-035F6E26A6A0}" name="Kategori" dataDxfId="41">
+    <tableColumn id="8" xr3:uid="{735DE14D-F3A8-4241-B953-035F6E26A6A0}" name="Kategori" dataDxfId="45">
       <calculatedColumnFormula>VLOOKUP(Table1[[#This Row],[SKU]],Table2[],3,FALSE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{ECD5AF4E-B3F4-41BB-B37B-443DEE5B7141}" name="Harga_Satuan" dataDxfId="40">
+    <tableColumn id="9" xr3:uid="{ECD5AF4E-B3F4-41BB-B37B-443DEE5B7141}" name="Harga_Satuan" dataDxfId="44">
       <calculatedColumnFormula>INDEX(Table2[Harga Jual],MATCH(Table1[[#This Row],[SKU]],Table2[SKU],0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{C465DBB9-4C64-4E93-9532-CB6D42B2E695}" name="HPP_Satuan" dataDxfId="39">
+    <tableColumn id="10" xr3:uid="{C465DBB9-4C64-4E93-9532-CB6D42B2E695}" name="HPP_Satuan" dataDxfId="43">
       <calculatedColumnFormula>VLOOKUP(Table1[[#This Row],[SKU]],Table2[],4,FALSE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{FBA65091-B8F3-4737-AD43-21E2351C753A}" name="Biaya_Kirim_Satuan" dataDxfId="38">
+    <tableColumn id="11" xr3:uid="{FBA65091-B8F3-4737-AD43-21E2351C753A}" name="Biaya_Kirim_Satuan" dataDxfId="42">
       <calculatedColumnFormula>INDEX(Table3[Biaya Kirim per Unit],MATCH(Table1[[#This Row],[Kota]],Table3[Kota],))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{236D1E61-E310-4595-8E7E-18D3E9DD1768}" name="Persentase_Diskon" dataDxfId="37" dataCellStyle="Percent">
+    <tableColumn id="12" xr3:uid="{236D1E61-E310-4595-8E7E-18D3E9DD1768}" name="Persentase_Diskon" dataDxfId="41" dataCellStyle="Percent">
       <calculatedColumnFormula>VLOOKUP(Table1[[#This Row],[Kode_Promo]],Table4[],2,FALSE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{CA31B10C-74E5-409B-A9BB-69CF31F44850}" name="Total_Pendapatan_Kotor" dataDxfId="36">
+    <tableColumn id="13" xr3:uid="{CA31B10C-74E5-409B-A9BB-69CF31F44850}" name="Total_Pendapatan_Kotor" dataDxfId="40">
       <calculatedColumnFormula>Table1[[#This Row],[Jumlah_Unit]]*Table1[[#This Row],[Harga_Satuan]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{3AE5F5BA-9CCD-4247-B4FB-CBB68DB0342F}" name="Potongan_Diskon" dataDxfId="35">
+    <tableColumn id="14" xr3:uid="{3AE5F5BA-9CCD-4247-B4FB-CBB68DB0342F}" name="Potongan_Diskon" dataDxfId="39">
       <calculatedColumnFormula>Table1[[#This Row],[Total_Pendapatan_Kotor]]*Table1[[#This Row],[Persentase_Diskon]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{83ED65EB-9A6F-4F9C-A403-5E4DEC52A650}" name="Total_Pendapatan_Bersih" dataDxfId="34">
+    <tableColumn id="15" xr3:uid="{83ED65EB-9A6F-4F9C-A403-5E4DEC52A650}" name="Total_Pendapatan_Bersih" dataDxfId="38">
       <calculatedColumnFormula>Table1[[#This Row],[Total_Pendapatan_Kotor]]-Table1[[#This Row],[Potongan_Diskon]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{C66B6AE0-9825-4E7F-9199-125CC56ED9A7}" name="Total_Biaya" dataDxfId="33">
+    <tableColumn id="16" xr3:uid="{C66B6AE0-9825-4E7F-9199-125CC56ED9A7}" name="Total_Biaya" dataDxfId="37">
       <calculatedColumnFormula>(Table1[[#This Row],[Jumlah_Unit]]*Table1[[#This Row],[HPP_Satuan]])+(Table1[[#This Row],[Jumlah_Unit]]*Table1[[#This Row],[Biaya_Kirim_Satuan]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{8448139B-E35F-403D-88B7-2B81687ED76E}" name="Laba_Kotor" dataDxfId="32">
+    <tableColumn id="17" xr3:uid="{8448139B-E35F-403D-88B7-2B81687ED76E}" name="Laba_Kotor" dataDxfId="36">
       <calculatedColumnFormula>Table1[[#This Row],[Total_Pendapatan_Bersih]]-Table1[[#This Row],[Total_Biaya]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="18" xr3:uid="{19F6E599-1DA2-4A17-B20A-85FAA9CAA88F}" name="Margin_Keuntungan" dataDxfId="31">
+    <tableColumn id="18" xr3:uid="{19F6E599-1DA2-4A17-B20A-85FAA9CAA88F}" name="Margin_Keuntungan" dataDxfId="35">
       <calculatedColumnFormula>Table1[[#This Row],[Laba_Kotor]]/Table1[[#This Row],[Total_Pendapatan_Bersih]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -16971,51 +20816,51 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{FDD45560-B6D3-41C6-AE2A-F8AD6BBACE68}" name="Table2" displayName="Table2" ref="A1:E6" totalsRowShown="0" headerRowDxfId="30" headerRowBorderDxfId="29" tableBorderDxfId="28" totalsRowBorderDxfId="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{FDD45560-B6D3-41C6-AE2A-F8AD6BBACE68}" name="Table2" displayName="Table2" ref="A1:E6" totalsRowShown="0" headerRowDxfId="34" headerRowBorderDxfId="33" tableBorderDxfId="32" totalsRowBorderDxfId="31">
   <autoFilter ref="A1:E6" xr:uid="{FDD45560-B6D3-41C6-AE2A-F8AD6BBACE68}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{8EB14854-7AF6-49A4-88AA-B3FDDCC42382}" name="SKU" dataDxfId="26"/>
-    <tableColumn id="2" xr3:uid="{5D2A612D-0698-4443-8219-30640E779857}" name="Nama Produk" dataDxfId="25"/>
-    <tableColumn id="3" xr3:uid="{A6103524-5795-4C97-B3D5-365566612506}" name="Kategori" dataDxfId="24"/>
-    <tableColumn id="4" xr3:uid="{E99EBFAC-0288-49E8-A2CE-BA8095F96A66}" name="HPP" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{3D2D3651-2CAB-4DFC-ABF1-674CCD068115}" name="Harga Jual" dataDxfId="22"/>
+    <tableColumn id="1" xr3:uid="{8EB14854-7AF6-49A4-88AA-B3FDDCC42382}" name="SKU" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{5D2A612D-0698-4443-8219-30640E779857}" name="Nama Produk" dataDxfId="29"/>
+    <tableColumn id="3" xr3:uid="{A6103524-5795-4C97-B3D5-365566612506}" name="Kategori" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{E99EBFAC-0288-49E8-A2CE-BA8095F96A66}" name="HPP" dataDxfId="27"/>
+    <tableColumn id="5" xr3:uid="{3D2D3651-2CAB-4DFC-ABF1-674CCD068115}" name="Harga Jual" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{10F71EA0-F0EC-4DFE-A2AB-43A6531E908A}" name="Table3" displayName="Table3" ref="A1:C5" totalsRowShown="0" headerRowBorderDxfId="21" tableBorderDxfId="20" totalsRowBorderDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{10F71EA0-F0EC-4DFE-A2AB-43A6531E908A}" name="Table3" displayName="Table3" ref="A1:C5" totalsRowShown="0" headerRowBorderDxfId="25" tableBorderDxfId="24" totalsRowBorderDxfId="23">
   <autoFilter ref="A1:C5" xr:uid="{10F71EA0-F0EC-4DFE-A2AB-43A6531E908A}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{0A45B6A5-0536-4D20-A5E2-7E4BD4BDCE05}" name="Kota" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{636D6F2C-8691-45F9-87EF-3C4669C8D4FE}" name="Wilayah" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{873955BF-A08E-404A-897B-9A4966E646E3}" name="Biaya Kirim per Unit" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{0A45B6A5-0536-4D20-A5E2-7E4BD4BDCE05}" name="Kota" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{636D6F2C-8691-45F9-87EF-3C4669C8D4FE}" name="Wilayah" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{873955BF-A08E-404A-897B-9A4966E646E3}" name="Biaya Kirim per Unit" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{DA8C010A-5D31-4A19-AF5C-380C4883E588}" name="Table4" displayName="Table4" ref="A1:C5" totalsRowShown="0" headerRowBorderDxfId="15" tableBorderDxfId="14" totalsRowBorderDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{DA8C010A-5D31-4A19-AF5C-380C4883E588}" name="Table4" displayName="Table4" ref="A1:C5" totalsRowShown="0" headerRowBorderDxfId="19" tableBorderDxfId="18" totalsRowBorderDxfId="17">
   <autoFilter ref="A1:C5" xr:uid="{DA8C010A-5D31-4A19-AF5C-380C4883E588}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{0FEAB7C0-9975-4BB3-97C0-65272C933D59}" name="Kode Promo" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{7268390E-5820-4F31-AA85-AF2D35552741}" name="Besaran Diskon" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{95D74BC3-E24F-46CD-A305-3DE4BBBB44D9}" name="Keterangan Syarat" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{0FEAB7C0-9975-4BB3-97C0-65272C933D59}" name="Kode Promo" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{7268390E-5820-4F31-AA85-AF2D35552741}" name="Besaran Diskon" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{95D74BC3-E24F-46CD-A305-3DE4BBBB44D9}" name="Keterangan Syarat" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{2D8BD81D-9F01-414B-A4EE-0F3E3758FAD8}" name="Table5" displayName="Table5" ref="A5:D12" totalsRowShown="0" headerRowDxfId="9" dataDxfId="7" headerRowBorderDxfId="8" tableBorderDxfId="6" totalsRowBorderDxfId="5" dataCellStyle="Percent">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{2D8BD81D-9F01-414B-A4EE-0F3E3758FAD8}" name="Table5" displayName="Table5" ref="A5:D12" totalsRowShown="0" headerRowDxfId="13" dataDxfId="11" headerRowBorderDxfId="12" tableBorderDxfId="10" totalsRowBorderDxfId="9" dataCellStyle="Percent">
   <autoFilter ref="A5:D12" xr:uid="{2D8BD81D-9F01-414B-A4EE-0F3E3758FAD8}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{C0DB13C7-69BD-4B04-AD37-A903E9718342}" name="Nomor Soal" dataDxfId="4" dataCellStyle="Percent"/>
-    <tableColumn id="2" xr3:uid="{0024CB6F-4755-4E2C-8351-AEB7946C3495}" name="Kategori Keterampilan" dataDxfId="3" dataCellStyle="Percent"/>
-    <tableColumn id="3" xr3:uid="{E54C8867-FE29-4C25-A0EC-89B409159D7E}" name="Instruksi Pengerjaan" dataDxfId="2" dataCellStyle="Percent"/>
-    <tableColumn id="4" xr3:uid="{2E3FF913-4ABB-4AED-AD44-A625313457B5}" name="Output yang Diharapkan" dataDxfId="1" dataCellStyle="Percent"/>
+    <tableColumn id="1" xr3:uid="{C0DB13C7-69BD-4B04-AD37-A903E9718342}" name="Nomor Soal" dataDxfId="8" dataCellStyle="Percent"/>
+    <tableColumn id="2" xr3:uid="{0024CB6F-4755-4E2C-8351-AEB7946C3495}" name="Kategori Keterampilan" dataDxfId="7" dataCellStyle="Percent"/>
+    <tableColumn id="3" xr3:uid="{E54C8867-FE29-4C25-A0EC-89B409159D7E}" name="Instruksi Pengerjaan" dataDxfId="6" dataCellStyle="Percent"/>
+    <tableColumn id="4" xr3:uid="{2E3FF913-4ABB-4AED-AD44-A625313457B5}" name="Output yang Diharapkan" dataDxfId="5" dataCellStyle="Percent"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -17317,11 +21162,13 @@
 </file>
 
 <file path=xl/timelineCaches/timelineCache1.xml><?xml version="1.0" encoding="utf-8"?>
-<timelineCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="xr10" name="NativeTimeline_Tanggal" xr10:uid="{28F9D2A4-44D1-4593-B4E9-45FA56935458}" sourceName="Tanggal">
+<timelineCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="xr10" name="NativeTimeline_Tanggal" xr10:uid="{AD52D45B-92ED-4481-B367-3B377E209546}" sourceName="Tanggal">
   <pivotTables>
     <pivotTable tabId="6" name="analisis"/>
+    <pivotTable tabId="6" name="PivotTable1"/>
   </pivotTables>
-  <state minimalRefreshVersion="6" lastRefreshVersion="6" pivotCacheId="241815905" filterType="unknown">
+  <state minimalRefreshVersion="6" lastRefreshVersion="6" pivotCacheId="241815905" filterType="dateBetween">
+    <selection startDate="2025-02-01T00:00:00" endDate="2025-07-31T00:00:00"/>
     <bounds startDate="2025-01-01T00:00:00" endDate="2027-01-01T00:00:00"/>
   </state>
 </timelineCacheDefinition>
@@ -17329,7 +21176,7 @@
 
 <file path=xl/timelines/timeline1.xml><?xml version="1.0" encoding="utf-8"?>
 <timelines xmlns="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
-  <timeline name="Tanggal" xr10:uid="{2B7B3C0E-C565-4667-BEEF-8C2A92940EF5}" cache="NativeTimeline_Tanggal" caption="Tanggal" level="2" selectionLevel="2" scrollPosition="2025-01-01T00:00:00"/>
+  <timeline name="Tanggal" xr10:uid="{9DA8BBED-2023-4092-AEF7-60DAB179E2FA}" cache="NativeTimeline_Tanggal" caption="Tanggal" level="2" selectionLevel="2" scrollPosition="2025-01-01T00:00:00" style="blue template"/>
 </timelines>
 </file>
 
@@ -51416,7 +55263,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:R501">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>$E2 &gt; 5</formula>
     </cfRule>
   </conditionalFormatting>
@@ -51698,17 +55545,21 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEB7F205-A472-48BE-8BFF-99A604B10656}">
-  <dimension ref="A3:C9"/>
+  <dimension ref="A3:G9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="21" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="21" width="21.5703125" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="16.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="41" t="s">
         <v>6</v>
       </c>
@@ -51718,83 +55569,111 @@
       <c r="C3" t="s">
         <v>594</v>
       </c>
+      <c r="F3" s="41" t="s">
+        <v>2</v>
+      </c>
+      <c r="G3" t="s">
+        <v>595</v>
+      </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>539</v>
       </c>
       <c r="B4" s="26">
-        <v>567000000</v>
+        <v>289800000</v>
       </c>
       <c r="C4" s="49">
-        <v>29.245275888133023</v>
+        <v>14.017054043839757</v>
+      </c>
+      <c r="F4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" s="26">
+        <v>167845000</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>534</v>
       </c>
       <c r="B5" s="26">
-        <v>2676000000</v>
+        <v>1260000000</v>
       </c>
       <c r="C5" s="49">
-        <v>22.367766203703731</v>
+        <v>10.844340277777777</v>
+      </c>
+      <c r="F5" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" s="26">
+        <v>111475000</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>536</v>
       </c>
       <c r="B6" s="26">
-        <v>510000000</v>
+        <v>261800000</v>
       </c>
       <c r="C6" s="49">
-        <v>24.156746031746</v>
+        <v>12.644491129785242</v>
+      </c>
+      <c r="F6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" s="26">
+        <v>234065000</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>541</v>
       </c>
       <c r="B7" s="26">
-        <v>1071000000</v>
+        <v>512400000</v>
       </c>
       <c r="C7" s="49">
-        <v>30.3317507558579</v>
+        <v>14.975907029478458</v>
+      </c>
+      <c r="F7" t="s">
+        <v>23</v>
+      </c>
+      <c r="G7" s="26">
+        <v>120440000</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>538</v>
       </c>
       <c r="B8" s="26">
-        <v>996200000</v>
+        <v>489600000</v>
       </c>
       <c r="C8" s="49">
-        <v>24.34109477124181</v>
+        <v>12.231413398692801</v>
+      </c>
+      <c r="F8" t="s">
+        <v>590</v>
+      </c>
+      <c r="G8" s="26">
+        <v>633825000</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>590</v>
       </c>
       <c r="B9" s="26">
-        <v>5820200000</v>
+        <v>2813600000</v>
       </c>
       <c r="C9" s="49">
-        <v>130.44263365068247</v>
+        <v>64.713205879574033</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId2"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{7E03D99C-DC04-49d9-9315-930204A7B6E9}">
-      <x15:timelineRefs>
-        <x15:timelineRef r:id="rId3"/>
-      </x15:timelineRefs>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
 
@@ -52247,5 +56126,18 @@
     <mergeCell ref="T8:X10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{A8765BA9-456A-4dab-B4F3-ACF838C121DE}">
+      <x14:slicerList>
+        <x14:slicer r:id="rId2"/>
+      </x14:slicerList>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{7E03D99C-DC04-49d9-9315-930204A7B6E9}">
+      <x15:timelineRefs>
+        <x15:timelineRef r:id="rId3"/>
+      </x15:timelineRefs>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
</xml_diff>